<commit_message>
docs: update optimization plans and organize utilities
</commit_message>
<xml_diff>
--- a/1-wiki-资料沉淀/业务调研事项记录.xlsx
+++ b/1-wiki-资料沉淀/业务调研事项记录.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29100" windowHeight="13380"/>
+    <workbookView windowHeight="16760"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -750,13 +750,11 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
+      <top/>
+      <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -768,7 +766,9 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -778,13 +778,13 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color auto="1"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -1037,7 +1037,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1059,17 +1059,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1439,289 +1433,289 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" ht="18" spans="1:7">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="4"/>
+      <c r="G2" s="3"/>
     </row>
     <row r="3" ht="229" spans="1:7">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" ht="300" spans="1:7">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="6"/>
+      <c r="G4" s="4"/>
     </row>
     <row r="5" ht="18" spans="1:7">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
     </row>
     <row r="6" ht="88" spans="1:7">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" ht="36" spans="1:7">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="6"/>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" ht="141" spans="1:7">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="6"/>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" ht="141" spans="1:7">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="6"/>
+      <c r="G9" s="4"/>
     </row>
     <row r="10" ht="53" spans="1:7">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="6"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="11" ht="36" spans="1:7">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="6"/>
+      <c r="G11" s="4"/>
     </row>
     <row r="12" ht="176" spans="1:7">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="6"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" ht="18" spans="1:7">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G13" s="6"/>
+      <c r="G13" s="4"/>
     </row>
-    <row r="14" ht="36" spans="1:7">
-      <c r="A14" s="9" t="s">
+    <row r="14" ht="36" spans="1:6">
+      <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="10"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="5"/>
     </row>
-    <row r="15" ht="408" customHeight="1" spans="1:7">
-      <c r="A15" s="9" t="s">
+    <row r="15" ht="408" customHeight="1" spans="1:6">
+      <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="10" t="s">
+      <c r="E15" s="4"/>
+      <c r="F15" s="5" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update research records and intake reference
</commit_message>
<xml_diff>
--- a/1-wiki-资料沉淀/业务调研事项记录.xlsx
+++ b/1-wiki-资料沉淀/业务调研事项记录.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16760"/>
+    <workbookView windowWidth="29100" windowHeight="13380"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="122">
   <si>
     <t>业务模块</t>
   </si>
@@ -36,6 +36,9 @@
   </si>
   <si>
     <t>事项类型</t>
+  </si>
+  <si>
+    <t>事项简述</t>
   </si>
   <si>
     <t>事项描述</t>
@@ -290,16 +293,16 @@
     <t>出货计划的提前期和展望期？是否有锁定期？临时需求怎么处理？</t>
   </si>
   <si>
-    <t>否</t>
-  </si>
-  <si>
-    <t>需要跟CRM确认</t>
+    <t>展望期是1周，准确率90%，每周五做下周的周出货计划，每日做更精准的修正</t>
   </si>
   <si>
     <t>补货最小批量</t>
   </si>
   <si>
     <t>每次流入成品罐是否需要灌满整罐？是否需要按整罐补货？如果封罐才能售卖，不能边进边出，封罐的水位线是否有要求？</t>
+  </si>
+  <si>
+    <t>没有硬性要求，但区分淡旺季：旺季为了加速库存周转和满足出货频率，可以低液位封罐售卖；淡季由于周转慢，一般是在92%以上的液位封罐</t>
   </si>
   <si>
     <t>库存计划锁定期</t>
@@ -322,6 +325,220 @@
 b. 按周维度汇总，输出展望期内每周的总补货量；
 c. 锁定期：当周总补货量和每日补货计划和生产端协同后进行锁定，锁定期内不再更新；如果出货计划或者销售计划有调整，只更新展望期内除了锁定期以外的补货计划
 d. 更新机制：次周周初更新下一个展望期内的补货计划，以上述方式滚动</t>
+  </si>
+  <si>
+    <t>成本分摊</t>
+  </si>
+  <si>
+    <t>批次管理</t>
+  </si>
+  <si>
+    <t>问题确认</t>
+  </si>
+  <si>
+    <t>工艺转化</t>
+  </si>
+  <si>
+    <t>每一批物料在各工艺产出的质量怎么获取？收率是怎么获取？</t>
+  </si>
+  <si>
+    <t>糖化罐和QC罐进出</t>
+  </si>
+  <si>
+    <t>12个糖化罐是同时排出还是依次排出？
+QC罐是同时进料还是依次进料？</t>
+  </si>
+  <si>
+    <t>流量</t>
+  </si>
+  <si>
+    <t>管道和设备是全流还是半流还是变化的？
+如果没有生产负荷调整，单位时间的流量是恒定的还是变化？
+管道和设备里面的压力是恒定的吗？
+在管道中的流量和在设备中的流量是一样的吗？</t>
+  </si>
+  <si>
+    <t>质检</t>
+  </si>
+  <si>
+    <t>任意流程中质检不合格的批次怎么处理？</t>
+  </si>
+  <si>
+    <t>批次状态</t>
+  </si>
+  <si>
+    <t>批次状态异常的含义是什么？异常如果不参与追溯会导致整体成本出现问题</t>
+  </si>
+  <si>
+    <t>设备有效容积</t>
+  </si>
+  <si>
+    <t>设备的有效容积怎么获取？
+有效容积是质量吗？流体密度怎么计算？</t>
+  </si>
+  <si>
+    <t>误差累计</t>
+  </si>
+  <si>
+    <t>如果每个批次以上一批次终点作为下一批次起点，而过程时间又根据某一时刻平均流量计算，则一次流量误差会沿后续所有窗口累积。停机、降负荷、仪表缺数或重新计算还可能改变已生成的批次边界。</t>
+  </si>
+  <si>
+    <t>第3层：投料批次</t>
+  </si>
+  <si>
+    <t>淀粉乳罐</t>
+  </si>
+  <si>
+    <t>投料口后的三个罐（溶粉罐、乳罐、接收罐）是否有必要建立批次？</t>
+  </si>
+  <si>
+    <t>投料批次连续</t>
+  </si>
+  <si>
+    <t>需要通过一些预警机制确保投料时连续使用同一批次直到该批次用完</t>
+  </si>
+  <si>
+    <t>平均流量</t>
+  </si>
+  <si>
+    <t>投料过程中取的质量流量计是取淀粉乳接收罐后的质量流量计吗？
+过程时间中取批次启动时质量流量计的平均流量：批次启动时间是按照投料开始时间算吗？平均流量是需要设定某段时间流量波动性下降到某一阈值再计算平均流量吗？</t>
+  </si>
+  <si>
+    <t>第4层：糖化批次</t>
+  </si>
+  <si>
+    <t>阀门切换</t>
+  </si>
+  <si>
+    <t>DCS进罐阀门切换记录编号：阀门切换是指由关到开或者由开到关的状态切换吗？</t>
+  </si>
+  <si>
+    <t>进入糖化批次重量</t>
+  </si>
+  <si>
+    <t>怎么计算即将进入糖化批次的体积或者重量？需要用体积关联上游批次</t>
+  </si>
+  <si>
+    <t>糖化罐进液顺序</t>
+  </si>
+  <si>
+    <t>糖化罐同一时间是否只有一个罐开放？即装满后才会开放下一个糖化罐</t>
+  </si>
+  <si>
+    <t>批次多对多</t>
+  </si>
+  <si>
+    <t>由于糖化罐的容积和上游每个批次的体积不能完全对齐，可能会导致上游批次进入不同的罐中，导致批次关联出现多对多的情况</t>
+  </si>
+  <si>
+    <t>状态缺失</t>
+  </si>
+  <si>
+    <t>状态字段可能缺了一个糖化中的状态</t>
+  </si>
+  <si>
+    <t>第5层：F42中间品批次</t>
+  </si>
+  <si>
+    <t>首批生成规则</t>
+  </si>
+  <si>
+    <t>当日首个批次的起始时间生成规则：首先找到当日所有糖化罐批次尾号为001的批次，并找到这些批次中出罐时间最早的出罐时间，作为当日首批的起始时间切片；
+后续批次生成规则，按照过程时间依次首尾相接的向后推导，直到次日最早的批次</t>
+  </si>
+  <si>
+    <t>批次构成和关联</t>
+  </si>
+  <si>
+    <t>批次构成以及和上游关联：在批次起始时间记录所有糖化罐的液位，在批次结束时间记录所有糖化罐的液位，计算所有液位差值，根据上游糖化罐出料批次计算当前批次所有的上游批次构成例如TH03-001（40吨）、TH04-002（35吨）、TH05-002（25吨）</t>
+  </si>
+  <si>
+    <t>向下游分离比例</t>
+  </si>
+  <si>
+    <t>分离比例是手动调整的吗？分离比例变化频率是什么？</t>
+  </si>
+  <si>
+    <t>下游总产出量</t>
+  </si>
+  <si>
+    <t>产出F42比例，是否有收率？</t>
+  </si>
+  <si>
+    <t>第6层：色谱分离</t>
+  </si>
+  <si>
+    <t>树脂</t>
+  </si>
+  <si>
+    <t>树脂的使用周期怎么定义？怎么折算成本？</t>
+  </si>
+  <si>
+    <t>色谱分离工艺前是有阀门吗？
+阀门状态的切换依据是什么？
+时间窗起点是否以阀门切换至开的时间计算？</t>
+  </si>
+  <si>
+    <t>第7层：色谱分离</t>
+  </si>
+  <si>
+    <t>滤板</t>
+  </si>
+  <si>
+    <t>人工更换的滤板成本怎么计算？</t>
+  </si>
+  <si>
+    <t>入口时间</t>
+  </si>
+  <si>
+    <t>DCS记录每批物料的入口时间，怎么判断每个批次的起点？</t>
+  </si>
+  <si>
+    <t>多批次的量</t>
+  </si>
+  <si>
+    <t>当前批次同时来源于两个批次第5和第6，怎么判断来源两个批次的量？</t>
+  </si>
+  <si>
+    <t>切割规则</t>
+  </si>
+  <si>
+    <t>切割规则中的2小时一个批次是依据什么设定的？</t>
+  </si>
+  <si>
+    <t>配方切换</t>
+  </si>
+  <si>
+    <t>配方切换是立刻完成的吗？即配方切换时刻就开始生产新配方的产品？</t>
+  </si>
+  <si>
+    <t>第8层：QC罐</t>
+  </si>
+  <si>
+    <t>质检不合格返流</t>
+  </si>
+  <si>
+    <t>质检不合格的液体会根据原因返流到对应工序？返回后的处理是什么？
+暂停其他的料的进入优先处理返流的不合格料，还是有其他隔离手段？</t>
+  </si>
+  <si>
+    <t>第9层：成品罐</t>
+  </si>
+  <si>
+    <t>返流到QC罐</t>
+  </si>
+  <si>
+    <t>残留的液体会返回QC罐，然后再质检再判断是否继续返流到其他工艺流程还是回到成本罐，返回QC罐的流程是什么？返回的QC罐未满是继续装新批次的糖还是先判断完质量，分配好后续去向再继续装新批次的液体？</t>
+  </si>
+  <si>
+    <t>第10.1层：小包装</t>
+  </si>
+  <si>
+    <t>小包装</t>
+  </si>
+  <si>
+    <t>对于使用果糖成品继续加工的小包装产品，是否只剩下了分装的过程？这部分批次应该增加到整个批次管理流程里</t>
   </si>
 </sst>
 </file>
@@ -708,7 +925,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -753,19 +970,6 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -787,6 +991,32 @@
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -913,7 +1143,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -925,34 +1155,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1037,7 +1267,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1053,17 +1283,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1404,17 +1649,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="17.6" outlineLevelCol="6"/>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="17.6" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="20.8333333333333" customWidth="1"/>
-    <col min="3" max="3" width="18.6666666666667" customWidth="1"/>
-    <col min="4" max="4" width="62.8333333333333" customWidth="1"/>
-    <col min="5" max="5" width="10.8333333333333" customWidth="1"/>
-    <col min="6" max="6" width="69.8333333333333" customWidth="1"/>
+    <col min="3" max="4" width="18.6666666666667" customWidth="1"/>
+    <col min="5" max="5" width="64.8583333333333" customWidth="1"/>
+    <col min="6" max="6" width="10.8333333333333" customWidth="1"/>
+    <col min="7" max="7" width="69.8333333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.35" spans="1:7">
+    <row r="1" ht="18.35" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1424,7 +1669,7 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -1433,291 +1678,922 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" ht="18" spans="1:7">
-      <c r="A2" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="2" ht="18" spans="1:8">
+      <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" ht="229" spans="1:7">
-      <c r="A3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" ht="229" spans="1:8">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="D3" s="3"/>
+      <c r="E3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="4"/>
-    </row>
-    <row r="4" ht="300" spans="1:7">
-      <c r="A4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="F3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" ht="300" spans="1:8">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="C4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="4"/>
-    </row>
-    <row r="5" ht="18" spans="1:7">
-      <c r="A5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="F4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" ht="18" spans="1:8">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" ht="88" spans="1:7">
-      <c r="A6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="C5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="F5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" ht="88" spans="1:8">
+      <c r="A6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" ht="36" spans="1:7">
-      <c r="A7" s="4" t="s">
+      <c r="D6" s="3"/>
+      <c r="E6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="F6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" ht="36" spans="1:8">
+      <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="B7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="5" t="s">
+      <c r="C7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="8"/>
+      <c r="E7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" ht="141" spans="1:7">
-      <c r="A8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="F7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" ht="141" spans="1:8">
+      <c r="A8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="4" t="s">
+      <c r="C8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" ht="141" spans="1:7">
-      <c r="A9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="4" t="s">
+      <c r="F8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" ht="141" spans="1:8">
+      <c r="A9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="5" t="s">
+      <c r="C9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" ht="53" spans="1:7">
-      <c r="A10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="F9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" ht="53" spans="1:8">
+      <c r="A10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="5" t="s">
+      <c r="C10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" ht="36" spans="1:7">
-      <c r="A11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="4" t="s">
+      <c r="F10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" ht="36" spans="1:8">
+      <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="5" t="s">
+      <c r="C11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="4"/>
-    </row>
-    <row r="12" ht="176" spans="1:7">
-      <c r="A12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="4" t="s">
+      <c r="F11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" ht="176" spans="1:8">
+      <c r="A12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="C12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" ht="18" spans="1:7">
-      <c r="A13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="F12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" ht="18" spans="1:8">
+      <c r="A13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="C13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" ht="36" spans="1:6">
-      <c r="A14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="4" t="s">
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" ht="36" spans="1:8">
+      <c r="A14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="5" t="s">
+      <c r="C14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="5"/>
-    </row>
-    <row r="15" ht="408" customHeight="1" spans="1:6">
-      <c r="A15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="F14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="5" t="s">
+    </row>
+    <row r="15" ht="408" customHeight="1" spans="1:8">
+      <c r="A15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="5" t="s">
+      <c r="C15" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="11" t="s">
         <v>52</v>
       </c>
+      <c r="F15" s="10"/>
+      <c r="G15" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" ht="18" spans="1:8">
+      <c r="A16" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" ht="36" spans="1:8">
+      <c r="A17" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" ht="71" spans="1:8">
+      <c r="A18" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" ht="36" spans="1:8">
+      <c r="A20" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" ht="36" spans="1:8">
+      <c r="A21" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+    </row>
+    <row r="22" ht="53" spans="1:8">
+      <c r="A22" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+    </row>
+    <row r="23" ht="18" spans="1:8">
+      <c r="A23" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" ht="71" spans="1:8">
+      <c r="A25" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" ht="36" spans="1:8">
+      <c r="A26" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" ht="36" spans="1:8">
+      <c r="A29" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="31" ht="88" spans="1:8">
+      <c r="A31" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" ht="71" spans="1:8">
+      <c r="A32" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+    </row>
+    <row r="36" ht="53" spans="1:8">
+      <c r="A36" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+    </row>
+    <row r="37" ht="18" spans="1:8">
+      <c r="A37" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="E37" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+    </row>
+    <row r="42" ht="36" spans="1:8">
+      <c r="A42" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="E42" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+    </row>
+    <row r="43" ht="53" spans="1:8">
+      <c r="A43" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="E43" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+    </row>
+    <row r="44" ht="36" spans="1:8">
+      <c r="A44" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="E44" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="F44" s="12"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="12"/>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="12"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="12"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" s="12"/>
+      <c r="B47" s="12"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="12"/>
+      <c r="H47" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: add cost allocation and process traceability materials
</commit_message>
<xml_diff>
--- a/1-wiki-资料沉淀/业务调研事项记录.xlsx
+++ b/1-wiki-资料沉淀/业务调研事项记录.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="131">
   <si>
     <t>业务模块</t>
   </si>
@@ -342,11 +342,19 @@
     <t>每一批物料在各工艺产出的质量怎么获取？收率是怎么获取？</t>
   </si>
   <si>
-    <t>糖化罐和QC罐进出</t>
-  </si>
-  <si>
-    <t>12个糖化罐是同时排出还是依次排出？
-QC罐是同时进料还是依次进料？</t>
+    <t>投料口和各罐进出方式</t>
+  </si>
+  <si>
+    <t>投料口数量是多少？
+12个糖化罐是同时进料还是依次进料？同时排出还是依次排出？依次是否有优先级？
+QC罐是同时进料还是依次进料？同时排出还是依次排出？依次是否有优先级？
+成品罐是同时进料还是依次进料？同时排出还是依次排出？依次是否有优先级？</t>
+  </si>
+  <si>
+    <t>投料口：一共8个，同时投料。
+糖化罐：依次进，依次排，DCS控制顺序
+QC罐：依次进，依次出，DCS控制顺序
+成品罐：依次进，依次出，DCS控制顺序</t>
   </si>
   <si>
     <t>流量</t>
@@ -448,10 +456,16 @@
 后续批次生成规则，按照过程时间依次首尾相接的向后推导，直到次日最早的批次</t>
   </si>
   <si>
+    <t>如果是糖化罐依次初，规则会出现变化</t>
+  </si>
+  <si>
     <t>批次构成和关联</t>
   </si>
   <si>
     <t>批次构成以及和上游关联：在批次起始时间记录所有糖化罐的液位，在批次结束时间记录所有糖化罐的液位，计算所有液位差值，根据上游糖化罐出料批次计算当前批次所有的上游批次构成例如TH03-001（40吨）、TH04-002（35吨）、TH05-002（25吨）</t>
+  </si>
+  <si>
+    <t>如果是糖化罐依次进，规则会出现变化</t>
   </si>
   <si>
     <t>向下游分离比例</t>
@@ -516,10 +530,10 @@
     <t>第8层：QC罐</t>
   </si>
   <si>
-    <t>质检不合格返流</t>
-  </si>
-  <si>
-    <t>质检不合格的液体会根据原因返流到对应工序？返回后的处理是什么？
+    <t>质检不合格冻结和返流</t>
+  </si>
+  <si>
+    <t>质检不合格的液体做冻结时是实物上的冻结吗？然后返流会根据原因返流到对应工序吗？返回后的处理是什么？
 暂停其他的料的进入优先处理返流的不合格料，还是有其他隔离手段？</t>
   </si>
   <si>
@@ -530,6 +544,24 @@
   </si>
   <si>
     <t>残留的液体会返回QC罐，然后再质检再判断是否继续返流到其他工艺流程还是回到成本罐，返回QC罐的流程是什么？返回的QC罐未满是继续装新批次的糖还是先判断完质量，分配好后续去向再继续装新批次的液体？</t>
+  </si>
+  <si>
+    <t>成品罐状态</t>
+  </si>
+  <si>
+    <t>进罐状态需要增加空罐和出货中</t>
+  </si>
+  <si>
+    <t>第10层：车次</t>
+  </si>
+  <si>
+    <t>签收状态</t>
+  </si>
+  <si>
+    <t>部分签收的含义是什么？实际会怎么签收</t>
+  </si>
+  <si>
+    <t>除了销售订单号外，还需要生成发货单号</t>
   </si>
   <si>
     <t>第10.1层：小包装</t>
@@ -1267,7 +1299,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1292,9 +1324,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1303,9 +1332,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1649,12 +1675,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="17.6" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="20.8333333333333" customWidth="1"/>
-    <col min="3" max="4" width="18.6666666666667" customWidth="1"/>
-    <col min="5" max="5" width="64.8583333333333" customWidth="1"/>
+    <col min="3" max="3" width="18.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="22.7333333333333" customWidth="1"/>
+    <col min="5" max="5" width="66.1083333333333" customWidth="1"/>
     <col min="6" max="6" width="10.8333333333333" customWidth="1"/>
     <col min="7" max="7" width="69.8333333333333" customWidth="1"/>
   </cols>
@@ -1801,7 +1828,7 @@
       <c r="C7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="8"/>
+      <c r="D7" s="5"/>
       <c r="E7" s="7" t="s">
         <v>28</v>
       </c>
@@ -1845,7 +1872,7 @@
       <c r="C9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="8"/>
+      <c r="D9" s="5"/>
       <c r="E9" s="7" t="s">
         <v>34</v>
       </c>
@@ -1867,7 +1894,7 @@
       <c r="C10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="8"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="7" t="s">
         <v>37</v>
       </c>
@@ -1940,7 +1967,7 @@
       <c r="F13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>47</v>
       </c>
       <c r="H13" s="3"/>
@@ -1967,633 +1994,699 @@
       </c>
     </row>
     <row r="15" ht="408" customHeight="1" spans="1:8">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="11" t="s">
+      <c r="D15" s="9"/>
+      <c r="E15" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="F15" s="10"/>
-      <c r="G15" s="11" t="s">
+      <c r="F15" s="9"/>
+      <c r="G15" s="10" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" ht="18" spans="1:8">
-      <c r="A16" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" s="12" t="s">
+      <c r="A16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="12" t="s">
+      <c r="C16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-    </row>
-    <row r="17" ht="36" spans="1:8">
-      <c r="A17" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B17" s="12" t="s">
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" ht="124" spans="1:8">
+      <c r="A17" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="12" t="s">
+      <c r="C17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="H17" s="3"/>
     </row>
     <row r="18" ht="71" spans="1:8">
-      <c r="A18" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18" s="12" t="s">
+      <c r="A18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="E18" s="13" t="s">
+      <c r="C18" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
+      <c r="E18" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="12" t="s">
+      <c r="A19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="12" t="s">
+      <c r="C19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
+      <c r="E19" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
     </row>
     <row r="20" ht="36" spans="1:8">
-      <c r="A20" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B20" s="12" t="s">
+      <c r="A20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" s="13" t="s">
+      <c r="C20" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
+      <c r="E20" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
     </row>
     <row r="21" ht="36" spans="1:8">
-      <c r="A21" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B21" s="12" t="s">
+      <c r="A21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="13" t="s">
+      <c r="C21" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
+      <c r="E21" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
     </row>
     <row r="22" ht="53" spans="1:8">
-      <c r="A22" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="12" t="s">
+      <c r="A22" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="E22" s="13" t="s">
+      <c r="C22" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
+      <c r="E22" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
     </row>
     <row r="23" ht="18" spans="1:8">
-      <c r="A23" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D23" s="12" t="s">
+      <c r="A23" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="C23" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
+      <c r="E23" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="E24" s="12" t="s">
+      <c r="A24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
+      <c r="E24" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
     </row>
     <row r="25" ht="71" spans="1:8">
-      <c r="A25" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="E25" s="13" t="s">
+      <c r="A25" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
+      <c r="E25" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
     </row>
     <row r="26" ht="36" spans="1:8">
-      <c r="A26" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D26" s="12" t="s">
+      <c r="A26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="C26" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
+      <c r="E26" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="E27" s="12" t="s">
+      <c r="A27" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
+      <c r="E27" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="E28" s="12" t="s">
+      <c r="A28" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
+      <c r="E28" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
     </row>
     <row r="29" ht="36" spans="1:8">
-      <c r="A29" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="E29" s="13" t="s">
+      <c r="A29" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
+      <c r="E29" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="E30" s="12" t="s">
+      <c r="A30" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
+      <c r="E30" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
     </row>
     <row r="31" ht="88" spans="1:8">
-      <c r="A31" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D31" s="12" t="s">
+      <c r="A31" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="C31" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
+      <c r="E31" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H31" s="3"/>
     </row>
     <row r="32" ht="71" spans="1:8">
-      <c r="A32" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D32" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
+      <c r="A32" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H32" s="3"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D33" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="E33" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
+      <c r="A33" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
     </row>
     <row r="34" spans="1:8">
-      <c r="A34" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
+      <c r="A34" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
     </row>
     <row r="35" spans="1:8">
-      <c r="A35" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D35" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="12"/>
+      <c r="A35" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
     </row>
     <row r="36" ht="53" spans="1:8">
-      <c r="A36" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D36" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="E36" s="13" t="s">
+      <c r="A36" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
+      <c r="C36" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
     </row>
     <row r="37" ht="18" spans="1:8">
-      <c r="A37" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
+      <c r="A37" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D38" s="12" t="s">
+      <c r="A38" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="E38" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
+      <c r="C38" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
     </row>
     <row r="39" spans="1:8">
-      <c r="A39" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D39" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="E39" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
+      <c r="A39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
     </row>
     <row r="40" spans="1:8">
-      <c r="A40" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D40" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="E40" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
+      <c r="A40" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C41" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D41" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="E41" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="12"/>
-    </row>
-    <row r="42" ht="36" spans="1:8">
-      <c r="A42" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C42" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D42" s="12" t="s">
+      <c r="A41" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D41" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E41" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F42" s="12"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="12"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" ht="53" spans="1:8">
+      <c r="A42" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
     </row>
     <row r="43" ht="53" spans="1:8">
-      <c r="A43" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="C43" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D43" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="F43" s="12"/>
-      <c r="G43" s="12"/>
-      <c r="H43" s="12"/>
-    </row>
-    <row r="44" ht="36" spans="1:8">
-      <c r="A44" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B44" s="12" t="s">
+      <c r="A43" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C44" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D44" s="12" t="s">
+      <c r="C43" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D43" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E44" s="13" t="s">
+      <c r="E43" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="12"/>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="12"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="12"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="12"/>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="12"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" ht="18" spans="1:8">
+      <c r="A44" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+    </row>
+    <row r="45" ht="18" spans="1:8">
+      <c r="A45" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" ht="18" spans="1:8">
+      <c r="A46" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" ht="36" spans="1:8">
+      <c r="A47" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" s="3"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="3"/>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: add batch cost calculation plan
</commit_message>
<xml_diff>
--- a/1-wiki-资料沉淀/业务调研事项记录.xlsx
+++ b/1-wiki-资料沉淀/业务调研事项记录.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="133">
   <si>
     <t>业务模块</t>
   </si>
@@ -342,6 +342,10 @@
     <t>每一批物料在各工艺产出的质量怎么获取？收率是怎么获取？</t>
   </si>
   <si>
+    <t>算出来
+来源QMS，LIMS</t>
+  </si>
+  <si>
     <t>投料口和各罐进出方式</t>
   </si>
   <si>
@@ -398,6 +402,9 @@
   </si>
   <si>
     <t>投料口后的三个罐（溶粉罐、乳罐、接收罐）是否有必要建立批次？</t>
+  </si>
+  <si>
+    <t>没必要</t>
   </si>
   <si>
     <t>投料批次连续</t>
@@ -2012,7 +2019,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" ht="18" spans="1:8">
+    <row r="16" ht="36" spans="1:8">
       <c r="A16" s="3" t="s">
         <v>54</v>
       </c>
@@ -2029,7 +2036,9 @@
         <v>58</v>
       </c>
       <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
+      <c r="G16" s="11" t="s">
+        <v>59</v>
+      </c>
       <c r="H16" s="3"/>
     </row>
     <row r="17" ht="124" spans="1:8">
@@ -2043,14 +2052,14 @@
         <v>56</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H17" s="3"/>
     </row>
@@ -2065,10 +2074,10 @@
         <v>56</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -2085,10 +2094,10 @@
         <v>56</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -2105,10 +2114,10 @@
         <v>56</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -2125,10 +2134,10 @@
         <v>56</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -2145,10 +2154,10 @@
         <v>56</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -2159,19 +2168,21 @@
         <v>54</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
+      <c r="G23" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="H23" s="3"/>
     </row>
     <row r="24" spans="1:8">
@@ -2179,16 +2190,16 @@
         <v>54</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -2199,16 +2210,16 @@
         <v>54</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -2219,16 +2230,16 @@
         <v>54</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -2239,16 +2250,16 @@
         <v>54</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -2259,16 +2270,16 @@
         <v>54</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -2279,16 +2290,16 @@
         <v>54</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -2299,16 +2310,16 @@
         <v>54</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -2319,20 +2330,20 @@
         <v>54</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H31" s="3"/>
     </row>
@@ -2341,20 +2352,20 @@
         <v>54</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H32" s="3"/>
     </row>
@@ -2363,16 +2374,16 @@
         <v>54</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -2383,16 +2394,16 @@
         <v>54</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -2403,16 +2414,16 @@
         <v>54</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -2423,16 +2434,16 @@
         <v>54</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -2443,16 +2454,16 @@
         <v>54</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -2463,16 +2474,16 @@
         <v>54</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -2483,16 +2494,16 @@
         <v>54</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -2503,16 +2514,16 @@
         <v>54</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -2523,16 +2534,16 @@
         <v>54</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -2543,16 +2554,16 @@
         <v>54</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -2563,16 +2574,16 @@
         <v>54</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -2583,16 +2594,16 @@
         <v>54</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -2603,16 +2614,16 @@
         <v>54</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -2623,16 +2634,16 @@
         <v>54</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
@@ -2643,16 +2654,16 @@
         <v>54</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>56</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>

</xml_diff>